<commit_message>
feat: corregir cronogramas públicos y aislar conectores
</commit_message>
<xml_diff>
--- a/Horarios/Colectivos/322-Canuelas/DomingoCanuelas.xlsx
+++ b/Horarios/Colectivos/322-Canuelas/DomingoCanuelas.xlsx
@@ -158,7 +158,7 @@
     <tableColumn id="1" name="Tipo"/>
     <tableColumn id="2" name="Formacion"/>
     <tableColumn id="3" name="Marcos Paz"/>
-    <tableColumn id="4" name="Las Heras"/>
+    <tableColumn id="4" name="General Las Heras"/>
     <tableColumn id="5" name="Cañuelas"/>
   </tableColumns>
 </table>
@@ -481,7 +481,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Las Heras</t>
+          <t>General Las Heras</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>135_337856-1</t>
+          <t>322 E · 04:20</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.1805555555555556</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.2284722222222222</v>
+        <v>0.20625</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.2798611111111111</v>
+        <v>0.2638888888888889</v>
       </c>
     </row>
     <row r="3">
@@ -519,17 +519,19 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>135_337857-1</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0.375</v>
+          <t>322 D · 07:14</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.3951388888888889</v>
+        <v>0.3013888888888889</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.4465277777777778</v>
+        <v>0.3631944444444444</v>
       </c>
     </row>
     <row r="4">
@@ -540,17 +542,17 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>135_337858-1</t>
+          <t>322 E · 12:20</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.5138888888888888</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.5618055555555556</v>
+        <v>0.54375</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.6131944444444445</v>
+        <v>0.6048611111111111</v>
       </c>
     </row>
     <row r="5">
@@ -559,10 +561,22 @@
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n"/>
-      <c r="E5" s="1" t="n"/>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>322 D · 15:14</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.6347222222222222</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.6965277777777777</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -674,7 +688,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B16" s="1" t="n"/>
       <c r="C16" s="1" t="n"/>
@@ -694,7 +708,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46264</v>
+        <v>46276</v>
       </c>
       <c r="B18" s="1" t="n"/>
       <c r="C18" s="1" t="n"/>
@@ -715,7 +729,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>https://www.argentina.gob.ar/sube/cuandosubo</t>
+          <t>https://moovitapp.com/index/es-419/transporte_p%C3%BAblico-line-322-Buenos_Aires-1602-855399-579299-11</t>
         </is>
       </c>
       <c r="B20" s="1" t="n"/>
@@ -737,7 +751,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>https://cuandosubo.sube.gob.ar/onebusaway-api-webapp/api/where</t>
+          <t>https://moovitapp.com/index/es-419/transporte_p%C3%BAblico-time-322-Buenos_Aires-1602-855399-579299-6997977-0</t>
         </is>
       </c>
       <c r="B22" s="1" t="n"/>
@@ -759,7 +773,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>Estimado</t>
         </is>
       </c>
       <c r="B24" s="1" t="n"/>

</xml_diff>